<commit_message>
docs: gongfa catalog - use full grade labels
</commit_message>
<xml_diff>
--- a/metadata/gongfa/catalog.xlsx
+++ b/metadata/gongfa/catalog.xlsx
@@ -594,7 +594,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>天高</t>
+          <t>天阶高级</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>地高</t>
+          <t>地阶高级</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>地高</t>
+          <t>地阶高级</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>地高</t>
+          <t>地阶高级</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>地中</t>
+          <t>地阶中级</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -5426,7 +5426,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -5762,7 +5762,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -5874,7 +5874,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -6103,7 +6103,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -6335,7 +6335,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -6569,7 +6569,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -6794,7 +6794,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -7118,7 +7118,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -7232,7 +7232,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -7342,7 +7342,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -8177,7 +8177,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -8529,7 +8529,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -8647,7 +8647,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -8941,7 +8941,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -9118,7 +9118,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -9475,7 +9475,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -9827,7 +9827,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -10004,7 +10004,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -10181,7 +10181,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -10382,7 +10382,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>地初</t>
+          <t>地阶初级</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -10703,7 +10703,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -10845,7 +10845,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -10987,7 +10987,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -11129,7 +11129,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -11268,7 +11268,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -11912,7 +11912,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -12029,7 +12029,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -12146,7 +12146,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -12263,7 +12263,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -12499,7 +12499,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -12615,7 +12615,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -12734,7 +12734,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -12965,7 +12965,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -13204,7 +13204,7 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -13432,7 +13432,7 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -13544,7 +13544,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -13775,7 +13775,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -13887,7 +13887,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -13999,7 +13999,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -14111,7 +14111,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -14223,7 +14223,7 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -14335,7 +14335,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -14449,7 +14449,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -14561,7 +14561,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -14673,7 +14673,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -14899,7 +14899,7 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -15011,7 +15011,7 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -15235,7 +15235,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -15347,7 +15347,7 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -15459,7 +15459,7 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -15571,7 +15571,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -15683,7 +15683,7 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -15795,7 +15795,7 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -15907,7 +15907,7 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
@@ -16021,7 +16021,7 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -16249,7 +16249,7 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
@@ -16361,7 +16361,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -16473,7 +16473,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -16587,7 +16587,7 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -16699,7 +16699,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -16817,7 +16817,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -16931,7 +16931,7 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
@@ -17043,7 +17043,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -17155,7 +17155,7 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
@@ -17267,7 +17267,7 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
@@ -17379,7 +17379,7 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
@@ -17495,7 +17495,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
@@ -17602,7 +17602,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -17711,7 +17711,7 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
@@ -17818,7 +17818,7 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -17931,7 +17931,7 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
@@ -18038,7 +18038,7 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
@@ -18145,7 +18145,7 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
@@ -18252,7 +18252,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
@@ -18472,7 +18472,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
@@ -18579,7 +18579,7 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
@@ -18686,7 +18686,7 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
@@ -18793,7 +18793,7 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
@@ -18906,7 +18906,7 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
@@ -19025,7 +19025,7 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
@@ -19135,7 +19135,7 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
@@ -19245,7 +19245,7 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
@@ -19361,7 +19361,7 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
@@ -19471,7 +19471,7 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
@@ -19700,7 +19700,7 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
@@ -19819,7 +19819,7 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
@@ -19938,7 +19938,7 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
@@ -20051,7 +20051,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
@@ -20176,7 +20176,7 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
@@ -20299,7 +20299,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
@@ -20418,7 +20418,7 @@
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
@@ -20544,7 +20544,7 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
@@ -20654,7 +20654,7 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
@@ -20770,7 +20770,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
@@ -20889,7 +20889,7 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
@@ -21011,7 +21011,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
@@ -21121,7 +21121,7 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
@@ -21231,7 +21231,7 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
@@ -21341,7 +21341,7 @@
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
@@ -21457,7 +21457,7 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
@@ -21570,7 +21570,7 @@
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
@@ -21683,7 +21683,7 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
@@ -21796,7 +21796,7 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
@@ -21914,7 +21914,7 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
@@ -22027,7 +22027,7 @@
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
@@ -22140,7 +22140,7 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
@@ -22253,7 +22253,7 @@
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
@@ -22376,7 +22376,7 @@
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
@@ -22489,7 +22489,7 @@
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
@@ -22602,7 +22602,7 @@
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
@@ -22720,7 +22720,7 @@
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
@@ -22833,7 +22833,7 @@
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
@@ -22946,7 +22946,7 @@
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
@@ -23059,7 +23059,7 @@
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
@@ -23177,7 +23177,7 @@
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
@@ -23295,7 +23295,7 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
@@ -23409,7 +23409,7 @@
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
@@ -23523,7 +23523,7 @@
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
@@ -23631,7 +23631,7 @@
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
@@ -23745,7 +23745,7 @@
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
@@ -23859,7 +23859,7 @@
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
@@ -23973,7 +23973,7 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
@@ -24086,7 +24086,7 @@
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
@@ -24199,7 +24199,7 @@
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
@@ -24312,7 +24312,7 @@
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
@@ -24425,7 +24425,7 @@
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
@@ -24538,7 +24538,7 @@
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
@@ -24645,7 +24645,7 @@
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr">
@@ -24763,7 +24763,7 @@
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
@@ -24876,7 +24876,7 @@
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
@@ -24989,7 +24989,7 @@
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
@@ -25107,7 +25107,7 @@
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
@@ -25220,7 +25220,7 @@
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
@@ -25338,7 +25338,7 @@
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
@@ -25451,7 +25451,7 @@
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
@@ -25564,7 +25564,7 @@
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
@@ -25677,7 +25677,7 @@
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
@@ -25795,7 +25795,7 @@
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
@@ -25908,7 +25908,7 @@
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
@@ -26026,7 +26026,7 @@
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
@@ -26139,7 +26139,7 @@
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
@@ -26257,7 +26257,7 @@
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
@@ -26370,7 +26370,7 @@
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
@@ -26482,7 +26482,7 @@
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
@@ -26594,7 +26594,7 @@
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
@@ -26780,7 +26780,7 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
@@ -26964,7 +26964,7 @@
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
@@ -27153,7 +27153,7 @@
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
@@ -27328,7 +27328,7 @@
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
@@ -27505,7 +27505,7 @@
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
@@ -27681,7 +27681,7 @@
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
@@ -27859,7 +27859,7 @@
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
@@ -28035,7 +28035,7 @@
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
@@ -28211,7 +28211,7 @@
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
@@ -28393,7 +28393,7 @@
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
@@ -28572,7 +28572,7 @@
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>玄高</t>
+          <t>玄阶高级</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
@@ -28779,7 +28779,7 @@
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
@@ -28886,7 +28886,7 @@
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
@@ -29017,7 +29017,7 @@
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
@@ -29145,7 +29145,7 @@
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
@@ -29288,7 +29288,7 @@
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
@@ -29428,7 +29428,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -29570,7 +29570,7 @@
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
@@ -29712,7 +29712,7 @@
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
@@ -29854,7 +29854,7 @@
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
@@ -29995,7 +29995,7 @@
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
@@ -30124,7 +30124,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -30253,7 +30253,7 @@
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
@@ -30382,7 +30382,7 @@
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
@@ -30511,7 +30511,7 @@
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
@@ -30640,7 +30640,7 @@
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
@@ -30768,7 +30768,7 @@
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
@@ -30926,7 +30926,7 @@
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
@@ -31044,7 +31044,7 @@
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
@@ -31166,7 +31166,7 @@
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
@@ -31279,7 +31279,7 @@
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
@@ -31396,7 +31396,7 @@
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
@@ -31506,7 +31506,7 @@
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
@@ -31618,7 +31618,7 @@
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
@@ -31730,7 +31730,7 @@
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
@@ -31842,7 +31842,7 @@
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
@@ -31954,7 +31954,7 @@
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
@@ -32070,7 +32070,7 @@
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
@@ -32182,7 +32182,7 @@
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
@@ -32294,7 +32294,7 @@
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
@@ -32406,7 +32406,7 @@
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
@@ -32518,7 +32518,7 @@
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
@@ -32630,7 +32630,7 @@
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
@@ -32742,7 +32742,7 @@
       </c>
       <c r="B265" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
@@ -32854,7 +32854,7 @@
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
@@ -32966,7 +32966,7 @@
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
@@ -33078,7 +33078,7 @@
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
@@ -33190,7 +33190,7 @@
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
@@ -33302,7 +33302,7 @@
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
@@ -33414,7 +33414,7 @@
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
@@ -33526,7 +33526,7 @@
       </c>
       <c r="B272" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
@@ -33638,7 +33638,7 @@
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
@@ -33750,7 +33750,7 @@
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
@@ -33862,7 +33862,7 @@
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
@@ -33974,7 +33974,7 @@
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
@@ -34088,7 +34088,7 @@
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
@@ -34200,7 +34200,7 @@
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
@@ -34312,7 +34312,7 @@
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
@@ -34424,7 +34424,7 @@
       </c>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
@@ -34536,7 +34536,7 @@
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
@@ -34648,7 +34648,7 @@
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
@@ -34760,7 +34760,7 @@
       </c>
       <c r="B283" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C283" s="2" t="inlineStr">
@@ -34872,7 +34872,7 @@
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
@@ -34984,7 +34984,7 @@
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
@@ -35102,7 +35102,7 @@
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
@@ -35214,7 +35214,7 @@
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
@@ -35326,7 +35326,7 @@
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
@@ -35433,7 +35433,7 @@
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
@@ -35540,7 +35540,7 @@
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
@@ -35647,7 +35647,7 @@
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
@@ -35758,7 +35758,7 @@
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
@@ -35865,7 +35865,7 @@
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
@@ -35976,7 +35976,7 @@
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
@@ -36083,7 +36083,7 @@
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
@@ -36190,7 +36190,7 @@
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
@@ -36297,7 +36297,7 @@
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
@@ -36404,7 +36404,7 @@
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
@@ -36514,7 +36514,7 @@
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
@@ -36621,7 +36621,7 @@
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
@@ -36728,7 +36728,7 @@
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
@@ -36835,7 +36835,7 @@
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
@@ -37055,7 +37055,7 @@
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
@@ -37165,7 +37165,7 @@
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
@@ -37275,7 +37275,7 @@
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
@@ -37385,7 +37385,7 @@
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
@@ -37495,7 +37495,7 @@
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
@@ -37605,7 +37605,7 @@
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
@@ -37715,7 +37715,7 @@
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
@@ -37828,7 +37828,7 @@
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
@@ -37942,7 +37942,7 @@
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
@@ -38052,7 +38052,7 @@
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
@@ -38162,7 +38162,7 @@
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
@@ -38272,7 +38272,7 @@
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
@@ -38382,7 +38382,7 @@
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
@@ -38492,7 +38492,7 @@
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
@@ -38611,7 +38611,7 @@
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
@@ -38721,7 +38721,7 @@
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
@@ -38834,7 +38834,7 @@
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
@@ -38947,7 +38947,7 @@
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
@@ -39060,7 +39060,7 @@
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
@@ -39173,7 +39173,7 @@
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
@@ -39286,7 +39286,7 @@
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
@@ -39393,7 +39393,7 @@
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
@@ -39500,7 +39500,7 @@
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
@@ -39618,7 +39618,7 @@
       </c>
       <c r="B327" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
@@ -39731,7 +39731,7 @@
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
@@ -39839,7 +39839,7 @@
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
@@ -39953,7 +39953,7 @@
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
@@ -40072,7 +40072,7 @@
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
@@ -40300,7 +40300,7 @@
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
@@ -40414,7 +40414,7 @@
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
@@ -40522,7 +40522,7 @@
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
@@ -40629,7 +40629,7 @@
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
@@ -40742,7 +40742,7 @@
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
@@ -40855,7 +40855,7 @@
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
@@ -40962,7 +40962,7 @@
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
@@ -41080,7 +41080,7 @@
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
@@ -41193,7 +41193,7 @@
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
@@ -41306,7 +41306,7 @@
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
@@ -41419,7 +41419,7 @@
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
@@ -41532,7 +41532,7 @@
       </c>
       <c r="B344" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
@@ -41650,7 +41650,7 @@
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
@@ -41757,7 +41757,7 @@
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
@@ -41870,7 +41870,7 @@
       </c>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
@@ -41983,7 +41983,7 @@
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
@@ -42096,7 +42096,7 @@
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
@@ -42209,7 +42209,7 @@
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
@@ -42322,7 +42322,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -42434,7 +42434,7 @@
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
@@ -42620,7 +42620,7 @@
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>玄中</t>
+          <t>玄阶中级</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
@@ -42807,7 +42807,7 @@
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
@@ -42946,7 +42946,7 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -43085,7 +43085,7 @@
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
@@ -43214,7 +43214,7 @@
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
@@ -43343,7 +43343,7 @@
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
@@ -43581,7 +43581,7 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
@@ -43693,7 +43693,7 @@
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
@@ -43805,7 +43805,7 @@
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
@@ -43917,7 +43917,7 @@
       </c>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
@@ -44029,7 +44029,7 @@
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
@@ -44136,7 +44136,7 @@
       </c>
       <c r="B365" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
@@ -44250,7 +44250,7 @@
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
@@ -44361,7 +44361,7 @@
       </c>
       <c r="B367" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
@@ -44468,7 +44468,7 @@
       </c>
       <c r="B368" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
@@ -44575,7 +44575,7 @@
       </c>
       <c r="B369" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
@@ -44682,7 +44682,7 @@
       </c>
       <c r="B370" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
@@ -44793,7 +44793,7 @@
       </c>
       <c r="B371" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
@@ -44900,7 +44900,7 @@
       </c>
       <c r="B372" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
@@ -45007,7 +45007,7 @@
       </c>
       <c r="B373" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
@@ -45114,7 +45114,7 @@
       </c>
       <c r="B374" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
@@ -45221,7 +45221,7 @@
       </c>
       <c r="B375" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
@@ -45335,7 +45335,7 @@
       </c>
       <c r="B376" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
@@ -45445,7 +45445,7 @@
       </c>
       <c r="B377" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
@@ -45555,7 +45555,7 @@
       </c>
       <c r="B378" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
@@ -45665,7 +45665,7 @@
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
@@ -45779,7 +45779,7 @@
       </c>
       <c r="B380" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
@@ -45893,7 +45893,7 @@
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
@@ -46007,7 +46007,7 @@
       </c>
       <c r="B382" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C382" s="2" t="inlineStr">
@@ -46121,7 +46121,7 @@
       </c>
       <c r="B383" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C383" s="2" t="inlineStr">
@@ -46234,7 +46234,7 @@
       </c>
       <c r="B384" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C384" s="2" t="inlineStr">
@@ -46341,7 +46341,7 @@
       </c>
       <c r="B385" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C385" s="2" t="inlineStr">
@@ -46448,7 +46448,7 @@
       </c>
       <c r="B386" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C386" s="2" t="inlineStr">
@@ -46561,7 +46561,7 @@
       </c>
       <c r="B387" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C387" s="2" t="inlineStr">
@@ -46674,7 +46674,7 @@
       </c>
       <c r="B388" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C388" s="2" t="inlineStr">
@@ -46787,7 +46787,7 @@
       </c>
       <c r="B389" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C389" s="2" t="inlineStr">
@@ -46900,7 +46900,7 @@
       </c>
       <c r="B390" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C390" s="2" t="inlineStr">
@@ -47013,7 +47013,7 @@
       </c>
       <c r="B391" s="2" t="inlineStr">
         <is>
-          <t>玄初</t>
+          <t>玄阶初级</t>
         </is>
       </c>
       <c r="C391" s="2" t="inlineStr">
@@ -47126,7 +47126,7 @@
       </c>
       <c r="B392" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C392" s="2" t="inlineStr">
@@ -47239,7 +47239,7 @@
       </c>
       <c r="B393" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C393" s="2" t="inlineStr">
@@ -47379,7 +47379,7 @@
       </c>
       <c r="B394" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C394" s="2" t="inlineStr">
@@ -47509,7 +47509,7 @@
       </c>
       <c r="B395" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C395" s="2" t="inlineStr">
@@ -47638,7 +47638,7 @@
       </c>
       <c r="B396" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C396" s="2" t="inlineStr">
@@ -47761,7 +47761,7 @@
       </c>
       <c r="B397" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C397" s="2" t="inlineStr">
@@ -47873,7 +47873,7 @@
       </c>
       <c r="B398" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C398" s="2" t="inlineStr">
@@ -47985,7 +47985,7 @@
       </c>
       <c r="B399" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C399" s="2" t="inlineStr">
@@ -48092,7 +48092,7 @@
       </c>
       <c r="B400" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C400" s="2" t="inlineStr">
@@ -48199,7 +48199,7 @@
       </c>
       <c r="B401" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C401" s="2" t="inlineStr">
@@ -48306,7 +48306,7 @@
       </c>
       <c r="B402" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C402" s="2" t="inlineStr">
@@ -48413,7 +48413,7 @@
       </c>
       <c r="B403" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C403" s="2" t="inlineStr">
@@ -48520,7 +48520,7 @@
       </c>
       <c r="B404" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C404" s="2" t="inlineStr">
@@ -48642,7 +48642,7 @@
       </c>
       <c r="B405" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C405" s="2" t="inlineStr">
@@ -48753,7 +48753,7 @@
       </c>
       <c r="B406" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C406" s="2" t="inlineStr">
@@ -48867,7 +48867,7 @@
       </c>
       <c r="B407" s="2" t="inlineStr">
         <is>
-          <t>黄高</t>
+          <t>黄阶高级</t>
         </is>
       </c>
       <c r="C407" s="2" t="inlineStr">
@@ -48974,7 +48974,7 @@
       </c>
       <c r="B408" s="2" t="inlineStr">
         <is>
-          <t>黄中</t>
+          <t>黄阶中级</t>
         </is>
       </c>
       <c r="C408" s="2" t="inlineStr">
@@ -49103,7 +49103,7 @@
       </c>
       <c r="B409" s="2" t="inlineStr">
         <is>
-          <t>黄中</t>
+          <t>黄阶中级</t>
         </is>
       </c>
       <c r="C409" s="2" t="inlineStr">
@@ -49333,7 +49333,7 @@
       </c>
       <c r="B410" s="2" t="inlineStr">
         <is>
-          <t>黄中</t>
+          <t>黄阶中级</t>
         </is>
       </c>
       <c r="C410" s="2" t="inlineStr">
@@ -49444,7 +49444,7 @@
       </c>
       <c r="B411" s="2" t="inlineStr">
         <is>
-          <t>黄中</t>
+          <t>黄阶中级</t>
         </is>
       </c>
       <c r="C411" s="2" t="inlineStr">
@@ -49551,7 +49551,7 @@
       </c>
       <c r="B412" s="2" t="inlineStr">
         <is>
-          <t>黄初</t>
+          <t>黄阶初级</t>
         </is>
       </c>
       <c r="C412" s="2" t="inlineStr">

</xml_diff>